<commit_message>
Update app.py and output files
</commit_message>
<xml_diff>
--- a/output/cv_jepang.xlsx
+++ b/output/cv_jepang.xlsx
@@ -1572,7 +1572,7 @@
       </c>
       <c r="C2" s="113" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D2" s="114" t="n"/>
@@ -1630,7 +1630,7 @@
       <c r="E5" s="125" t="n"/>
       <c r="F5" s="126" t="inlineStr">
         <is>
-          <t>ギナ</t>
+          <t>アカ・セブン</t>
         </is>
       </c>
       <c r="G5" s="124" t="n"/>
@@ -1658,7 +1658,7 @@
       <c r="E6" s="121" t="n"/>
       <c r="F6" s="131" t="inlineStr">
         <is>
-          <t>gina</t>
+          <t>jaka sembung</t>
         </is>
       </c>
       <c r="G6" s="120" t="n"/>

</xml_diff>